<commit_message>
feat(data): validate Kentucky workbook and generate county data at build time
Adds key/source_label/data_year to the Data_Dictionary, a build step that
writes counties.json, fields.json and a downloadable CSV, labels.ts as the
single owner of source wording, and fictional sample communities. Removes
the hand-kept county CSV now that it is generated from the workbook.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/NourishScope_Kentucky_County_Dataset_v1.0.xlsx
+++ b/data/NourishScope_Kentucky_County_Dataset_v1.0.xlsx
@@ -655,8 +655,6 @@
       <c r="V2" t="n">
         <v>1</v>
       </c>
-      <c r="W2" t="inlineStr"/>
-      <c r="X2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -679,7 +677,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
       <c r="F3" t="n">
         <v>1</v>
       </c>
@@ -731,8 +728,6 @@
       <c r="V3" t="n">
         <v>0</v>
       </c>
-      <c r="W3" t="inlineStr"/>
-      <c r="X3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -755,7 +750,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr"/>
       <c r="F4" t="n">
         <v>0</v>
       </c>
@@ -795,7 +789,6 @@
       <c r="R4" t="n">
         <v>2.33</v>
       </c>
-      <c r="S4" t="inlineStr"/>
       <c r="T4" t="n">
         <v>18</v>
       </c>
@@ -805,8 +798,6 @@
       <c r="V4" t="n">
         <v>0</v>
       </c>
-      <c r="W4" t="inlineStr"/>
-      <c r="X4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -829,7 +820,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E5" t="inlineStr"/>
       <c r="F5" t="n">
         <v>1</v>
       </c>
@@ -869,7 +859,6 @@
       <c r="R5" t="n">
         <v>0.01</v>
       </c>
-      <c r="S5" t="inlineStr"/>
       <c r="T5" t="n">
         <v>14</v>
       </c>
@@ -879,8 +868,6 @@
       <c r="V5" t="n">
         <v>0</v>
       </c>
-      <c r="W5" t="inlineStr"/>
-      <c r="X5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -903,7 +890,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E6" t="inlineStr"/>
       <c r="F6" t="n">
         <v>0</v>
       </c>
@@ -955,8 +941,6 @@
       <c r="V6" t="n">
         <v>2</v>
       </c>
-      <c r="W6" t="inlineStr"/>
-      <c r="X6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1023,7 +1007,6 @@
       <c r="R7" t="n">
         <v>0.92</v>
       </c>
-      <c r="S7" t="inlineStr"/>
       <c r="T7" t="n">
         <v>12</v>
       </c>
@@ -1033,8 +1016,6 @@
       <c r="V7" t="n">
         <v>1</v>
       </c>
-      <c r="W7" t="inlineStr"/>
-      <c r="X7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1113,8 +1094,6 @@
       <c r="V8" t="n">
         <v>0</v>
       </c>
-      <c r="W8" t="inlineStr"/>
-      <c r="X8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1137,7 +1116,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E9" t="inlineStr"/>
       <c r="F9" t="n">
         <v>1</v>
       </c>
@@ -1189,8 +1167,6 @@
       <c r="V9" t="n">
         <v>0</v>
       </c>
-      <c r="W9" t="inlineStr"/>
-      <c r="X9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1213,7 +1189,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E10" t="inlineStr"/>
       <c r="F10" t="n">
         <v>1</v>
       </c>
@@ -1253,7 +1228,6 @@
       <c r="R10" t="n">
         <v>12.26</v>
       </c>
-      <c r="S10" t="inlineStr"/>
       <c r="T10" t="n">
         <v>21</v>
       </c>
@@ -1263,8 +1237,6 @@
       <c r="V10" t="n">
         <v>0</v>
       </c>
-      <c r="W10" t="inlineStr"/>
-      <c r="X10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1343,8 +1315,6 @@
       <c r="V11" t="n">
         <v>0</v>
       </c>
-      <c r="W11" t="inlineStr"/>
-      <c r="X11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1367,7 +1337,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E12" t="inlineStr"/>
       <c r="F12" t="n">
         <v>0</v>
       </c>
@@ -1419,8 +1388,6 @@
       <c r="V12" t="n">
         <v>1</v>
       </c>
-      <c r="W12" t="inlineStr"/>
-      <c r="X12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1443,7 +1410,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E13" t="inlineStr"/>
       <c r="F13" t="n">
         <v>1</v>
       </c>
@@ -1483,7 +1449,6 @@
       <c r="R13" t="n">
         <v>0.23</v>
       </c>
-      <c r="S13" t="inlineStr"/>
       <c r="T13" t="n">
         <v>7</v>
       </c>
@@ -1493,8 +1458,6 @@
       <c r="V13" t="n">
         <v>0</v>
       </c>
-      <c r="W13" t="inlineStr"/>
-      <c r="X13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1573,8 +1536,6 @@
       <c r="V14" t="n">
         <v>0</v>
       </c>
-      <c r="W14" t="inlineStr"/>
-      <c r="X14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1597,7 +1558,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E15" t="inlineStr"/>
       <c r="F15" t="n">
         <v>0</v>
       </c>
@@ -1649,8 +1609,6 @@
       <c r="V15" t="n">
         <v>0</v>
       </c>
-      <c r="W15" t="inlineStr"/>
-      <c r="X15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1673,7 +1631,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E16" t="inlineStr"/>
       <c r="F16" t="n">
         <v>1</v>
       </c>
@@ -1725,8 +1682,6 @@
       <c r="V16" t="n">
         <v>0</v>
       </c>
-      <c r="W16" t="inlineStr"/>
-      <c r="X16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1749,7 +1704,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E17" t="inlineStr"/>
       <c r="F17" t="n">
         <v>1</v>
       </c>
@@ -1789,7 +1743,6 @@
       <c r="R17" t="n">
         <v>4.83</v>
       </c>
-      <c r="S17" t="inlineStr"/>
       <c r="T17" t="n">
         <v>13</v>
       </c>
@@ -1799,8 +1752,6 @@
       <c r="V17" t="n">
         <v>0</v>
       </c>
-      <c r="W17" t="inlineStr"/>
-      <c r="X17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1823,7 +1774,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E18" t="inlineStr"/>
       <c r="F18" t="n">
         <v>0</v>
       </c>
@@ -1875,8 +1825,6 @@
       <c r="V18" t="n">
         <v>0</v>
       </c>
-      <c r="W18" t="inlineStr"/>
-      <c r="X18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1899,7 +1847,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E19" t="inlineStr"/>
       <c r="F19" t="n">
         <v>0</v>
       </c>
@@ -1951,8 +1898,6 @@
       <c r="V19" t="n">
         <v>0</v>
       </c>
-      <c r="W19" t="inlineStr"/>
-      <c r="X19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1975,7 +1920,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E20" t="inlineStr"/>
       <c r="F20" t="n">
         <v>1</v>
       </c>
@@ -2027,8 +1971,6 @@
       <c r="V20" t="n">
         <v>0</v>
       </c>
-      <c r="W20" t="inlineStr"/>
-      <c r="X20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2051,7 +1993,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
       <c r="F21" t="n">
         <v>1</v>
       </c>
@@ -2091,7 +2032,6 @@
       <c r="R21" t="n">
         <v>3.35</v>
       </c>
-      <c r="S21" t="inlineStr"/>
       <c r="T21" t="n">
         <v>6</v>
       </c>
@@ -2101,8 +2041,6 @@
       <c r="V21" t="n">
         <v>0</v>
       </c>
-      <c r="W21" t="inlineStr"/>
-      <c r="X21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2125,7 +2063,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
       <c r="F22" t="n">
         <v>0</v>
       </c>
@@ -2165,7 +2102,6 @@
       <c r="R22" t="n">
         <v>0</v>
       </c>
-      <c r="S22" t="inlineStr"/>
       <c r="T22" t="n">
         <v>20</v>
       </c>
@@ -2175,8 +2111,6 @@
       <c r="V22" t="n">
         <v>0</v>
       </c>
-      <c r="W22" t="inlineStr"/>
-      <c r="X22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2255,8 +2189,6 @@
       <c r="V23" t="n">
         <v>0</v>
       </c>
-      <c r="W23" t="inlineStr"/>
-      <c r="X23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2335,8 +2267,6 @@
       <c r="V24" t="n">
         <v>0</v>
       </c>
-      <c r="W24" t="inlineStr"/>
-      <c r="X24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2359,7 +2289,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E25" t="inlineStr"/>
       <c r="F25" t="n">
         <v>1</v>
       </c>
@@ -2411,8 +2340,6 @@
       <c r="V25" t="n">
         <v>1</v>
       </c>
-      <c r="W25" t="inlineStr"/>
-      <c r="X25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2491,8 +2418,6 @@
       <c r="V26" t="n">
         <v>1</v>
       </c>
-      <c r="W26" t="inlineStr"/>
-      <c r="X26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2571,8 +2496,6 @@
       <c r="V27" t="n">
         <v>0</v>
       </c>
-      <c r="W27" t="inlineStr"/>
-      <c r="X27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2639,7 +2562,6 @@
       <c r="R28" t="n">
         <v>1.09</v>
       </c>
-      <c r="S28" t="inlineStr"/>
       <c r="T28" t="n">
         <v>12</v>
       </c>
@@ -2649,8 +2571,6 @@
       <c r="V28" t="n">
         <v>0</v>
       </c>
-      <c r="W28" t="inlineStr"/>
-      <c r="X28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2673,7 +2593,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E29" t="inlineStr"/>
       <c r="F29" t="n">
         <v>0</v>
       </c>
@@ -2713,7 +2632,6 @@
       <c r="R29" t="n">
         <v>4.76</v>
       </c>
-      <c r="S29" t="inlineStr"/>
       <c r="T29" t="n">
         <v>9</v>
       </c>
@@ -2723,8 +2641,6 @@
       <c r="V29" t="n">
         <v>1</v>
       </c>
-      <c r="W29" t="inlineStr"/>
-      <c r="X29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2791,7 +2707,6 @@
       <c r="R30" t="n">
         <v>0.8</v>
       </c>
-      <c r="S30" t="inlineStr"/>
       <c r="T30" t="n">
         <v>14</v>
       </c>
@@ -2801,8 +2716,6 @@
       <c r="V30" t="n">
         <v>0</v>
       </c>
-      <c r="W30" t="inlineStr"/>
-      <c r="X30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2825,7 +2738,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E31" t="inlineStr"/>
       <c r="F31" t="n">
         <v>1</v>
       </c>
@@ -2877,8 +2789,6 @@
       <c r="V31" t="n">
         <v>0</v>
       </c>
-      <c r="W31" t="inlineStr"/>
-      <c r="X31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -2945,7 +2855,6 @@
       <c r="R32" t="n">
         <v>2.02</v>
       </c>
-      <c r="S32" t="inlineStr"/>
       <c r="T32" t="n">
         <v>13</v>
       </c>
@@ -2955,8 +2864,6 @@
       <c r="V32" t="n">
         <v>0</v>
       </c>
-      <c r="W32" t="inlineStr"/>
-      <c r="X32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -3023,7 +2930,6 @@
       <c r="R33" t="n">
         <v>0</v>
       </c>
-      <c r="S33" t="inlineStr"/>
       <c r="T33" t="n">
         <v>9</v>
       </c>
@@ -3033,8 +2939,6 @@
       <c r="V33" t="n">
         <v>0</v>
       </c>
-      <c r="W33" t="inlineStr"/>
-      <c r="X33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -3113,8 +3017,6 @@
       <c r="V34" t="n">
         <v>0</v>
       </c>
-      <c r="W34" t="inlineStr"/>
-      <c r="X34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -3137,7 +3039,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E35" t="inlineStr"/>
       <c r="F35" t="n">
         <v>1</v>
       </c>
@@ -3189,8 +3090,6 @@
       <c r="V35" t="n">
         <v>5</v>
       </c>
-      <c r="W35" t="inlineStr"/>
-      <c r="X35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -3269,8 +3168,6 @@
       <c r="V36" t="n">
         <v>0</v>
       </c>
-      <c r="W36" t="inlineStr"/>
-      <c r="X36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -3349,8 +3246,6 @@
       <c r="V37" t="n">
         <v>1</v>
       </c>
-      <c r="W37" t="inlineStr"/>
-      <c r="X37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -3373,7 +3268,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
         <v>0</v>
       </c>
@@ -3425,8 +3319,6 @@
       <c r="V38" t="n">
         <v>1</v>
       </c>
-      <c r="W38" t="inlineStr"/>
-      <c r="X38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -3449,7 +3341,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
         <v>0</v>
       </c>
@@ -3489,7 +3380,6 @@
       <c r="R39" t="n">
         <v>0.03</v>
       </c>
-      <c r="S39" t="inlineStr"/>
       <c r="T39" t="n">
         <v>10</v>
       </c>
@@ -3499,8 +3389,6 @@
       <c r="V39" t="n">
         <v>0</v>
       </c>
-      <c r="W39" t="inlineStr"/>
-      <c r="X39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -3523,7 +3411,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
         <v>1</v>
       </c>
@@ -3563,7 +3450,6 @@
       <c r="R40" t="n">
         <v>0</v>
       </c>
-      <c r="S40" t="inlineStr"/>
       <c r="T40" t="n">
         <v>11</v>
       </c>
@@ -3573,8 +3459,6 @@
       <c r="V40" t="n">
         <v>0</v>
       </c>
-      <c r="W40" t="inlineStr"/>
-      <c r="X40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -3641,7 +3525,6 @@
       <c r="R41" t="n">
         <v>0</v>
       </c>
-      <c r="S41" t="inlineStr"/>
       <c r="T41" t="n">
         <v>13</v>
       </c>
@@ -3651,8 +3534,6 @@
       <c r="V41" t="n">
         <v>0</v>
       </c>
-      <c r="W41" t="inlineStr"/>
-      <c r="X41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -3675,7 +3556,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
         <v>1</v>
       </c>
@@ -3715,7 +3595,6 @@
       <c r="R42" t="n">
         <v>2.32</v>
       </c>
-      <c r="S42" t="inlineStr"/>
       <c r="T42" t="n">
         <v>22</v>
       </c>
@@ -3725,8 +3604,6 @@
       <c r="V42" t="n">
         <v>0</v>
       </c>
-      <c r="W42" t="inlineStr"/>
-      <c r="X42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -3749,7 +3626,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
         <v>0</v>
       </c>
@@ -3801,8 +3677,6 @@
       <c r="V43" t="n">
         <v>0</v>
       </c>
-      <c r="W43" t="inlineStr"/>
-      <c r="X43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -3825,7 +3699,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E44" t="inlineStr"/>
       <c r="F44" t="n">
         <v>0</v>
       </c>
@@ -3877,8 +3750,6 @@
       <c r="V44" t="n">
         <v>0</v>
       </c>
-      <c r="W44" t="inlineStr"/>
-      <c r="X44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -3945,7 +3816,6 @@
       <c r="R45" t="n">
         <v>4.2</v>
       </c>
-      <c r="S45" t="inlineStr"/>
       <c r="T45" t="n">
         <v>11</v>
       </c>
@@ -3955,8 +3825,6 @@
       <c r="V45" t="n">
         <v>0</v>
       </c>
-      <c r="W45" t="inlineStr"/>
-      <c r="X45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4035,8 +3903,6 @@
       <c r="V46" t="n">
         <v>0</v>
       </c>
-      <c r="W46" t="inlineStr"/>
-      <c r="X46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4059,7 +3925,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E47" t="inlineStr"/>
       <c r="F47" t="n">
         <v>0</v>
       </c>
@@ -4099,7 +3964,6 @@
       <c r="R47" t="n">
         <v>4.98</v>
       </c>
-      <c r="S47" t="inlineStr"/>
       <c r="T47" t="n">
         <v>8</v>
       </c>
@@ -4109,8 +3973,6 @@
       <c r="V47" t="n">
         <v>0</v>
       </c>
-      <c r="W47" t="inlineStr"/>
-      <c r="X47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4133,7 +3995,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E48" t="inlineStr"/>
       <c r="F48" t="n">
         <v>1</v>
       </c>
@@ -4185,8 +4046,6 @@
       <c r="V48" t="n">
         <v>1</v>
       </c>
-      <c r="W48" t="inlineStr"/>
-      <c r="X48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4265,8 +4124,6 @@
       <c r="V49" t="n">
         <v>0</v>
       </c>
-      <c r="W49" t="inlineStr"/>
-      <c r="X49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -4289,7 +4146,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E50" t="inlineStr"/>
       <c r="F50" t="n">
         <v>0</v>
       </c>
@@ -4341,8 +4197,6 @@
       <c r="V50" t="n">
         <v>0</v>
       </c>
-      <c r="W50" t="inlineStr"/>
-      <c r="X50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -4421,8 +4275,6 @@
       <c r="V51" t="n">
         <v>0</v>
       </c>
-      <c r="W51" t="inlineStr"/>
-      <c r="X51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -4445,7 +4297,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E52" t="inlineStr"/>
       <c r="F52" t="n">
         <v>0</v>
       </c>
@@ -4497,8 +4348,6 @@
       <c r="V52" t="n">
         <v>0</v>
       </c>
-      <c r="W52" t="inlineStr"/>
-      <c r="X52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -4521,7 +4370,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E53" t="inlineStr"/>
       <c r="F53" t="n">
         <v>1</v>
       </c>
@@ -4561,7 +4409,6 @@
       <c r="R53" t="n">
         <v>1.17</v>
       </c>
-      <c r="S53" t="inlineStr"/>
       <c r="T53" t="n">
         <v>21</v>
       </c>
@@ -4571,8 +4418,6 @@
       <c r="V53" t="n">
         <v>0</v>
       </c>
-      <c r="W53" t="inlineStr"/>
-      <c r="X53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -4595,7 +4440,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E54" t="inlineStr"/>
       <c r="F54" t="n">
         <v>0</v>
       </c>
@@ -4635,7 +4479,6 @@
       <c r="R54" t="n">
         <v>1.25</v>
       </c>
-      <c r="S54" t="inlineStr"/>
       <c r="T54" t="n">
         <v>3</v>
       </c>
@@ -4645,8 +4488,6 @@
       <c r="V54" t="n">
         <v>0</v>
       </c>
-      <c r="W54" t="inlineStr"/>
-      <c r="X54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -4669,7 +4510,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E55" t="inlineStr"/>
       <c r="F55" t="n">
         <v>0</v>
       </c>
@@ -4721,8 +4561,6 @@
       <c r="V55" t="n">
         <v>0</v>
       </c>
-      <c r="W55" t="inlineStr"/>
-      <c r="X55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -4789,7 +4627,6 @@
       <c r="R56" t="n">
         <v>3.7</v>
       </c>
-      <c r="S56" t="inlineStr"/>
       <c r="T56" t="n">
         <v>19</v>
       </c>
@@ -4799,8 +4636,6 @@
       <c r="V56" t="n">
         <v>0</v>
       </c>
-      <c r="W56" t="inlineStr"/>
-      <c r="X56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -4823,7 +4658,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E57" t="inlineStr"/>
       <c r="F57" t="n">
         <v>1</v>
       </c>
@@ -4875,8 +4709,6 @@
       <c r="V57" t="n">
         <v>6</v>
       </c>
-      <c r="W57" t="inlineStr"/>
-      <c r="X57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -4899,7 +4731,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E58" t="inlineStr"/>
       <c r="F58" t="n">
         <v>1</v>
       </c>
@@ -4951,8 +4782,6 @@
       <c r="V58" t="n">
         <v>0</v>
       </c>
-      <c r="W58" t="inlineStr"/>
-      <c r="X58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -5031,8 +4860,6 @@
       <c r="V59" t="n">
         <v>0</v>
       </c>
-      <c r="W59" t="inlineStr"/>
-      <c r="X59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -5055,7 +4882,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E60" t="inlineStr"/>
       <c r="F60" t="n">
         <v>1</v>
       </c>
@@ -5107,8 +4933,6 @@
       <c r="V60" t="n">
         <v>1</v>
       </c>
-      <c r="W60" t="inlineStr"/>
-      <c r="X60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -5187,8 +5011,6 @@
       <c r="V61" t="n">
         <v>0</v>
       </c>
-      <c r="W61" t="inlineStr"/>
-      <c r="X61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -5267,8 +5089,6 @@
       <c r="V62" t="n">
         <v>0</v>
       </c>
-      <c r="W62" t="inlineStr"/>
-      <c r="X62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -5291,7 +5111,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E63" t="inlineStr"/>
       <c r="F63" t="n">
         <v>1</v>
       </c>
@@ -5331,7 +5150,6 @@
       <c r="R63" t="n">
         <v>6.75</v>
       </c>
-      <c r="S63" t="inlineStr"/>
       <c r="T63" t="n">
         <v>15</v>
       </c>
@@ -5341,8 +5159,6 @@
       <c r="V63" t="n">
         <v>0</v>
       </c>
-      <c r="W63" t="inlineStr"/>
-      <c r="X63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -5421,8 +5237,6 @@
       <c r="V64" t="n">
         <v>0</v>
       </c>
-      <c r="W64" t="inlineStr"/>
-      <c r="X64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -5489,7 +5303,6 @@
       <c r="R65" t="n">
         <v>5.72</v>
       </c>
-      <c r="S65" t="inlineStr"/>
       <c r="T65" t="n">
         <v>20</v>
       </c>
@@ -5499,8 +5312,6 @@
       <c r="V65" t="n">
         <v>0</v>
       </c>
-      <c r="W65" t="inlineStr"/>
-      <c r="X65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -5567,7 +5378,6 @@
       <c r="R66" t="n">
         <v>0.01</v>
       </c>
-      <c r="S66" t="inlineStr"/>
       <c r="T66" t="n">
         <v>12</v>
       </c>
@@ -5577,8 +5387,6 @@
       <c r="V66" t="n">
         <v>0</v>
       </c>
-      <c r="W66" t="inlineStr"/>
-      <c r="X66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -5657,8 +5465,6 @@
       <c r="V67" t="n">
         <v>0</v>
       </c>
-      <c r="W67" t="inlineStr"/>
-      <c r="X67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -5737,8 +5543,6 @@
       <c r="V68" t="n">
         <v>1</v>
       </c>
-      <c r="W68" t="inlineStr"/>
-      <c r="X68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -5817,8 +5621,6 @@
       <c r="V69" t="n">
         <v>0</v>
       </c>
-      <c r="W69" t="inlineStr"/>
-      <c r="X69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -5897,8 +5699,6 @@
       <c r="V70" t="n">
         <v>0</v>
       </c>
-      <c r="W70" t="inlineStr"/>
-      <c r="X70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -5921,7 +5721,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E71" t="inlineStr"/>
       <c r="F71" t="n">
         <v>1</v>
       </c>
@@ -5973,8 +5772,6 @@
       <c r="V71" t="n">
         <v>0</v>
       </c>
-      <c r="W71" t="inlineStr"/>
-      <c r="X71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -5997,7 +5794,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E72" t="inlineStr"/>
       <c r="F72" t="n">
         <v>0</v>
       </c>
@@ -6049,8 +5845,6 @@
       <c r="V72" t="n">
         <v>0</v>
       </c>
-      <c r="W72" t="inlineStr"/>
-      <c r="X72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -6073,7 +5867,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E73" t="inlineStr"/>
       <c r="F73" t="n">
         <v>0</v>
       </c>
@@ -6113,7 +5906,6 @@
       <c r="R73" t="n">
         <v>1.03</v>
       </c>
-      <c r="S73" t="inlineStr"/>
       <c r="T73" t="n">
         <v>8</v>
       </c>
@@ -6123,8 +5915,6 @@
       <c r="V73" t="n">
         <v>0</v>
       </c>
-      <c r="W73" t="inlineStr"/>
-      <c r="X73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -6147,7 +5937,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E74" t="inlineStr"/>
       <c r="F74" t="n">
         <v>1</v>
       </c>
@@ -6199,8 +5988,6 @@
       <c r="V74" t="n">
         <v>0</v>
       </c>
-      <c r="W74" t="inlineStr"/>
-      <c r="X74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -6279,8 +6066,6 @@
       <c r="V75" t="n">
         <v>0</v>
       </c>
-      <c r="W75" t="inlineStr"/>
-      <c r="X75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -6303,7 +6088,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E76" t="inlineStr"/>
       <c r="F76" t="n">
         <v>1</v>
       </c>
@@ -6343,7 +6127,6 @@
       <c r="R76" t="n">
         <v>1.03</v>
       </c>
-      <c r="S76" t="inlineStr"/>
       <c r="T76" t="n">
         <v>11</v>
       </c>
@@ -6353,8 +6136,6 @@
       <c r="V76" t="n">
         <v>0</v>
       </c>
-      <c r="W76" t="inlineStr"/>
-      <c r="X76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -6433,8 +6214,6 @@
       <c r="V77" t="n">
         <v>1</v>
       </c>
-      <c r="W77" t="inlineStr"/>
-      <c r="X77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -6501,7 +6280,6 @@
       <c r="R78" t="n">
         <v>1.45</v>
       </c>
-      <c r="S78" t="inlineStr"/>
       <c r="T78" t="n">
         <v>17</v>
       </c>
@@ -6511,8 +6289,6 @@
       <c r="V78" t="n">
         <v>0</v>
       </c>
-      <c r="W78" t="inlineStr"/>
-      <c r="X78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -6535,7 +6311,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E79" t="inlineStr"/>
       <c r="F79" t="n">
         <v>0</v>
       </c>
@@ -6587,8 +6362,6 @@
       <c r="V79" t="n">
         <v>1</v>
       </c>
-      <c r="W79" t="inlineStr"/>
-      <c r="X79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -6611,7 +6384,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E80" t="inlineStr"/>
       <c r="F80" t="n">
         <v>0</v>
       </c>
@@ -6663,8 +6435,6 @@
       <c r="V80" t="n">
         <v>0</v>
       </c>
-      <c r="W80" t="inlineStr"/>
-      <c r="X80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -6743,8 +6513,6 @@
       <c r="V81" t="n">
         <v>0</v>
       </c>
-      <c r="W81" t="inlineStr"/>
-      <c r="X81" t="inlineStr"/>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -6767,7 +6535,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E82" t="inlineStr"/>
       <c r="F82" t="n">
         <v>0</v>
       </c>
@@ -6819,8 +6586,6 @@
       <c r="V82" t="n">
         <v>0</v>
       </c>
-      <c r="W82" t="inlineStr"/>
-      <c r="X82" t="inlineStr"/>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -6843,7 +6608,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E83" t="inlineStr"/>
       <c r="F83" t="n">
         <v>1</v>
       </c>
@@ -6895,8 +6659,6 @@
       <c r="V83" t="n">
         <v>1</v>
       </c>
-      <c r="W83" t="inlineStr"/>
-      <c r="X83" t="inlineStr"/>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -6963,7 +6725,6 @@
       <c r="R84" t="n">
         <v>0.28</v>
       </c>
-      <c r="S84" t="inlineStr"/>
       <c r="T84" t="n">
         <v>11</v>
       </c>
@@ -6973,8 +6734,6 @@
       <c r="V84" t="n">
         <v>0</v>
       </c>
-      <c r="W84" t="inlineStr"/>
-      <c r="X84" t="inlineStr"/>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -6997,7 +6756,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr"/>
       <c r="F85" t="n">
         <v>0</v>
       </c>
@@ -7049,8 +6807,6 @@
       <c r="V85" t="n">
         <v>0</v>
       </c>
-      <c r="W85" t="inlineStr"/>
-      <c r="X85" t="inlineStr"/>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -7117,7 +6873,6 @@
       <c r="R86" t="n">
         <v>0.48</v>
       </c>
-      <c r="S86" t="inlineStr"/>
       <c r="T86" t="n">
         <v>8</v>
       </c>
@@ -7127,8 +6882,6 @@
       <c r="V86" t="n">
         <v>1</v>
       </c>
-      <c r="W86" t="inlineStr"/>
-      <c r="X86" t="inlineStr"/>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -7207,8 +6960,6 @@
       <c r="V87" t="n">
         <v>0</v>
       </c>
-      <c r="W87" t="inlineStr"/>
-      <c r="X87" t="inlineStr"/>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -7287,8 +7038,6 @@
       <c r="V88" t="n">
         <v>0</v>
       </c>
-      <c r="W88" t="inlineStr"/>
-      <c r="X88" t="inlineStr"/>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -7367,8 +7116,6 @@
       <c r="V89" t="n">
         <v>0</v>
       </c>
-      <c r="W89" t="inlineStr"/>
-      <c r="X89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -7391,7 +7138,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E90" t="inlineStr"/>
       <c r="F90" t="n">
         <v>0</v>
       </c>
@@ -7443,8 +7189,6 @@
       <c r="V90" t="n">
         <v>0</v>
       </c>
-      <c r="W90" t="inlineStr"/>
-      <c r="X90" t="inlineStr"/>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -7467,7 +7211,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E91" t="inlineStr"/>
       <c r="F91" t="n">
         <v>1</v>
       </c>
@@ -7519,8 +7262,6 @@
       <c r="V91" t="n">
         <v>0</v>
       </c>
-      <c r="W91" t="inlineStr"/>
-      <c r="X91" t="inlineStr"/>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -7587,7 +7328,6 @@
       <c r="R92" t="n">
         <v>0.3</v>
       </c>
-      <c r="S92" t="inlineStr"/>
       <c r="T92" t="n">
         <v>5</v>
       </c>
@@ -7597,8 +7337,6 @@
       <c r="V92" t="n">
         <v>0</v>
       </c>
-      <c r="W92" t="inlineStr"/>
-      <c r="X92" t="inlineStr"/>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -7621,7 +7359,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E93" t="inlineStr"/>
       <c r="F93" t="n">
         <v>0</v>
       </c>
@@ -7661,7 +7398,6 @@
       <c r="R93" t="n">
         <v>2.88</v>
       </c>
-      <c r="S93" t="inlineStr"/>
       <c r="T93" t="n">
         <v>27</v>
       </c>
@@ -7671,8 +7407,6 @@
       <c r="V93" t="n">
         <v>1</v>
       </c>
-      <c r="W93" t="inlineStr"/>
-      <c r="X93" t="inlineStr"/>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -7695,7 +7429,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E94" t="inlineStr"/>
       <c r="F94" t="n">
         <v>1</v>
       </c>
@@ -7747,8 +7480,6 @@
       <c r="V94" t="n">
         <v>0</v>
       </c>
-      <c r="W94" t="inlineStr"/>
-      <c r="X94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -7771,7 +7502,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E95" t="inlineStr"/>
       <c r="F95" t="n">
         <v>0</v>
       </c>
@@ -7811,7 +7541,6 @@
       <c r="R95" t="n">
         <v>4.45</v>
       </c>
-      <c r="S95" t="inlineStr"/>
       <c r="T95" t="n">
         <v>13</v>
       </c>
@@ -7821,8 +7550,6 @@
       <c r="V95" t="n">
         <v>1</v>
       </c>
-      <c r="W95" t="inlineStr"/>
-      <c r="X95" t="inlineStr"/>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -7889,7 +7616,6 @@
       <c r="R96" t="n">
         <v>1.4</v>
       </c>
-      <c r="S96" t="inlineStr"/>
       <c r="T96" t="n">
         <v>8</v>
       </c>
@@ -7899,8 +7625,6 @@
       <c r="V96" t="n">
         <v>0</v>
       </c>
-      <c r="W96" t="inlineStr"/>
-      <c r="X96" t="inlineStr"/>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -7923,7 +7647,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E97" t="inlineStr"/>
       <c r="F97" t="n">
         <v>1</v>
       </c>
@@ -7963,7 +7686,6 @@
       <c r="R97" t="n">
         <v>0.2</v>
       </c>
-      <c r="S97" t="inlineStr"/>
       <c r="T97" t="n">
         <v>10</v>
       </c>
@@ -7973,8 +7695,6 @@
       <c r="V97" t="n">
         <v>1</v>
       </c>
-      <c r="W97" t="inlineStr"/>
-      <c r="X97" t="inlineStr"/>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -8053,8 +7773,6 @@
       <c r="V98" t="n">
         <v>1</v>
       </c>
-      <c r="W98" t="inlineStr"/>
-      <c r="X98" t="inlineStr"/>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -8133,8 +7851,6 @@
       <c r="V99" t="n">
         <v>0</v>
       </c>
-      <c r="W99" t="inlineStr"/>
-      <c r="X99" t="inlineStr"/>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -8213,8 +7929,6 @@
       <c r="V100" t="n">
         <v>0</v>
       </c>
-      <c r="W100" t="inlineStr"/>
-      <c r="X100" t="inlineStr"/>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -8293,8 +8007,6 @@
       <c r="V101" t="n">
         <v>1</v>
       </c>
-      <c r="W101" t="inlineStr"/>
-      <c r="X101" t="inlineStr"/>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -8361,7 +8073,6 @@
       <c r="R102" t="n">
         <v>29.35</v>
       </c>
-      <c r="S102" t="inlineStr"/>
       <c r="T102" t="n">
         <v>2</v>
       </c>
@@ -8371,8 +8082,6 @@
       <c r="V102" t="n">
         <v>0</v>
       </c>
-      <c r="W102" t="inlineStr"/>
-      <c r="X102" t="inlineStr"/>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -8451,8 +8160,6 @@
       <c r="V103" t="n">
         <v>0</v>
       </c>
-      <c r="W103" t="inlineStr"/>
-      <c r="X103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -8531,8 +8238,6 @@
       <c r="V104" t="n">
         <v>0</v>
       </c>
-      <c r="W104" t="inlineStr"/>
-      <c r="X104" t="inlineStr"/>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -8611,8 +8316,6 @@
       <c r="V105" t="n">
         <v>0</v>
       </c>
-      <c r="W105" t="inlineStr"/>
-      <c r="X105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -8635,7 +8338,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E106" t="inlineStr"/>
       <c r="F106" t="n">
         <v>1</v>
       </c>
@@ -8687,8 +8389,6 @@
       <c r="V106" t="n">
         <v>0</v>
       </c>
-      <c r="W106" t="inlineStr"/>
-      <c r="X106" t="inlineStr"/>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -8711,7 +8411,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E107" t="inlineStr"/>
       <c r="F107" t="n">
         <v>1</v>
       </c>
@@ -8763,8 +8462,6 @@
       <c r="V107" t="n">
         <v>0</v>
       </c>
-      <c r="W107" t="inlineStr"/>
-      <c r="X107" t="inlineStr"/>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -8787,7 +8484,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E108" t="inlineStr"/>
       <c r="F108" t="n">
         <v>0</v>
       </c>
@@ -8827,7 +8523,6 @@
       <c r="R108" t="n">
         <v>6.78</v>
       </c>
-      <c r="S108" t="inlineStr"/>
       <c r="T108" t="n">
         <v>21</v>
       </c>
@@ -8837,8 +8532,6 @@
       <c r="V108" t="n">
         <v>1</v>
       </c>
-      <c r="W108" t="inlineStr"/>
-      <c r="X108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -8861,7 +8554,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E109" t="inlineStr"/>
       <c r="F109" t="n">
         <v>1</v>
       </c>
@@ -8901,7 +8593,6 @@
       <c r="R109" t="n">
         <v>0</v>
       </c>
-      <c r="S109" t="inlineStr"/>
       <c r="T109" t="n">
         <v>12</v>
       </c>
@@ -8911,8 +8602,6 @@
       <c r="V109" t="n">
         <v>0</v>
       </c>
-      <c r="W109" t="inlineStr"/>
-      <c r="X109" t="inlineStr"/>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -8935,7 +8624,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E110" t="inlineStr"/>
       <c r="F110" t="n">
         <v>0</v>
       </c>
@@ -8987,8 +8675,6 @@
       <c r="V110" t="n">
         <v>0</v>
       </c>
-      <c r="W110" t="inlineStr"/>
-      <c r="X110" t="inlineStr"/>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -9011,7 +8697,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E111" t="inlineStr"/>
       <c r="F111" t="n">
         <v>0</v>
       </c>
@@ -9063,8 +8748,6 @@
       <c r="V111" t="n">
         <v>0</v>
       </c>
-      <c r="W111" t="inlineStr"/>
-      <c r="X111" t="inlineStr"/>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -9087,7 +8770,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E112" t="inlineStr"/>
       <c r="F112" t="n">
         <v>1</v>
       </c>
@@ -9127,7 +8809,6 @@
       <c r="R112" t="n">
         <v>1.6</v>
       </c>
-      <c r="S112" t="inlineStr"/>
       <c r="T112" t="n">
         <v>15</v>
       </c>
@@ -9137,8 +8818,6 @@
       <c r="V112" t="n">
         <v>0</v>
       </c>
-      <c r="W112" t="inlineStr"/>
-      <c r="X112" t="inlineStr"/>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -9161,7 +8840,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E113" t="inlineStr"/>
       <c r="F113" t="n">
         <v>0</v>
       </c>
@@ -9201,7 +8879,6 @@
       <c r="R113" t="n">
         <v>0</v>
       </c>
-      <c r="S113" t="inlineStr"/>
       <c r="T113" t="n">
         <v>6</v>
       </c>
@@ -9211,8 +8888,6 @@
       <c r="V113" t="n">
         <v>0</v>
       </c>
-      <c r="W113" t="inlineStr"/>
-      <c r="X113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -9235,7 +8910,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E114" t="inlineStr"/>
       <c r="F114" t="n">
         <v>0</v>
       </c>
@@ -9287,8 +8961,6 @@
       <c r="V114" t="n">
         <v>0</v>
       </c>
-      <c r="W114" t="inlineStr"/>
-      <c r="X114" t="inlineStr"/>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -9311,7 +8983,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E115" t="inlineStr"/>
       <c r="F115" t="n">
         <v>1</v>
       </c>
@@ -9363,8 +9034,6 @@
       <c r="V115" t="n">
         <v>3</v>
       </c>
-      <c r="W115" t="inlineStr"/>
-      <c r="X115" t="inlineStr"/>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -9387,7 +9056,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E116" t="inlineStr"/>
       <c r="F116" t="n">
         <v>0</v>
       </c>
@@ -9439,8 +9107,6 @@
       <c r="V116" t="n">
         <v>0</v>
       </c>
-      <c r="W116" t="inlineStr"/>
-      <c r="X116" t="inlineStr"/>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -9507,7 +9173,6 @@
       <c r="R117" t="n">
         <v>9.85</v>
       </c>
-      <c r="S117" t="inlineStr"/>
       <c r="T117" t="n">
         <v>27</v>
       </c>
@@ -9517,8 +9182,6 @@
       <c r="V117" t="n">
         <v>0</v>
       </c>
-      <c r="W117" t="inlineStr"/>
-      <c r="X117" t="inlineStr"/>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -9541,7 +9204,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E118" t="inlineStr"/>
       <c r="F118" t="n">
         <v>0</v>
       </c>
@@ -9593,8 +9255,6 @@
       <c r="V118" t="n">
         <v>0</v>
       </c>
-      <c r="W118" t="inlineStr"/>
-      <c r="X118" t="inlineStr"/>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -9673,8 +9333,6 @@
       <c r="V119" t="n">
         <v>0</v>
       </c>
-      <c r="W119" t="inlineStr"/>
-      <c r="X119" t="inlineStr"/>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -9741,7 +9399,6 @@
       <c r="R120" t="n">
         <v>2.69</v>
       </c>
-      <c r="S120" t="inlineStr"/>
       <c r="T120" t="n">
         <v>14</v>
       </c>
@@ -9751,8 +9408,6 @@
       <c r="V120" t="n">
         <v>0</v>
       </c>
-      <c r="W120" t="inlineStr"/>
-      <c r="X120" t="inlineStr"/>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -9775,7 +9430,6 @@
           <t>No</t>
         </is>
       </c>
-      <c r="E121" t="inlineStr"/>
       <c r="F121" t="n">
         <v>1</v>
       </c>
@@ -9827,8 +9481,6 @@
       <c r="V121" t="n">
         <v>3</v>
       </c>
-      <c r="W121" t="inlineStr"/>
-      <c r="X121" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -9841,7 +9493,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -9877,6 +9529,21 @@
           <t>status</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>key</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>source_label</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>data_year</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -9904,6 +9571,16 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>county_name</t>
+        </is>
+      </c>
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -9931,6 +9608,16 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>fips</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -9958,6 +9645,16 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>state</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>U.S. Census Bureau</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -9985,6 +9682,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>appalachian</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>ARC</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -10012,6 +9724,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>arc_status</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>ARC</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>FY2027</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -10039,6 +9766,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>metro_nonmetro</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -10066,6 +9808,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>population</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>Census ACS 5-year</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>2020–2024</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -10093,6 +9850,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>total_households</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>Census ACS 5-year</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>2020–2024</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -10120,6 +9892,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>snap_households</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Census ACS 5-year</t>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>2020–2024</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -10147,6 +9934,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>snap_household_pct</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Census ACS 5-year</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2020–2024</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -10174,6 +9976,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>poverty_rate</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -10201,6 +10018,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>child_poverty_rate</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -10228,6 +10060,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>persistent_poverty</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2017–2021</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -10255,6 +10102,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>median_household_income</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -10282,6 +10144,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>diabetes_pct</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>CDC PLACES</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -10309,6 +10186,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>obesity_pct</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>CDC PLACES</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -10336,6 +10228,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>high_bp_pct</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>CDC PLACES</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2021</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -10363,6 +10270,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>low_income_low_access_pct</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2019</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -10390,6 +10312,21 @@
           <t>Filled (78 of 120)</t>
         </is>
       </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>grocery_stores_per_1000</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -10417,6 +10354,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>snap_retailers</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -10444,6 +10396,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>farmers_markets</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -10471,6 +10438,21 @@
           <t>Filled</t>
         </is>
       </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>farmers_markets_snap</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>USDA ERS Food Environment Atlas</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2018</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -10498,6 +10480,16 @@
           <t>User enters in app</t>
         </is>
       </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>households_served</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>User-entered</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -10523,6 +10515,16 @@
       <c r="E25" s="2" t="inlineStr">
         <is>
           <t>User enters in app</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>cost_per_household</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>User-entered</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(copy): remove dashes, show Not entered/Not applicable, label the health score 2021-2022
</commit_message>
<xml_diff>
--- a/data/NourishScope_Kentucky_County_Dataset_v1.0.xlsx
+++ b/data/NourishScope_Kentucky_County_Dataset_v1.0.xlsx
@@ -9820,7 +9820,7 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2020–2024</t>
+          <t>2020-2024</t>
         </is>
       </c>
     </row>
@@ -9862,7 +9862,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2020–2024</t>
+          <t>2020-2024</t>
         </is>
       </c>
     </row>
@@ -9904,7 +9904,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2020–2024</t>
+          <t>2020-2024</t>
         </is>
       </c>
     </row>
@@ -9946,7 +9946,7 @@
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>2020–2024</t>
+          <t>2020-2024</t>
         </is>
       </c>
     </row>
@@ -10047,7 +10047,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>Persistent-poverty county, 2017–21 (1 = yes)</t>
+          <t>Persistent-poverty county, 2017-21 (1 = yes)</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -10072,7 +10072,7 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>2017–2021</t>
+          <t>2017-2021</t>
         </is>
       </c>
     </row>

</xml_diff>